<commit_message>
changed column name to have more generalized AI names
</commit_message>
<xml_diff>
--- a/results_all_thermostat.xlsx
+++ b/results_all_thermostat.xlsx
@@ -468,17 +468,17 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Claude Judgment</t>
+          <t>AI Judgment</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>Claude Judgment Reasoning</t>
+          <t>AI Judgment Reasoning</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>Claude Confidence</t>
+          <t>AI Confidence</t>
         </is>
       </c>
     </row>

</xml_diff>